<commit_message>
create figma pages (patient and doctors)
</commit_message>
<xml_diff>
--- a/Week_4/HealthCare Plus/Capstone Timesheet_Ripal Patel.xlsx
+++ b/Week_4/HealthCare Plus/Capstone Timesheet_Ripal Patel.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="43">
   <si>
     <t>Week_1</t>
   </si>
@@ -137,6 +137,9 @@
   </si>
   <si>
     <t>Prototyping pages</t>
+  </si>
+  <si>
+    <t>Add pages for patient, Doctors</t>
   </si>
 </sst>
 </file>
@@ -2319,9 +2322,15 @@
     </row>
     <row r="51">
       <c r="A51" s="32"/>
-      <c r="B51" s="33"/>
-      <c r="C51" s="34"/>
-      <c r="D51" s="35"/>
+      <c r="B51" s="33" t="s">
+        <v>42</v>
+      </c>
+      <c r="C51" s="34">
+        <v>46062.0</v>
+      </c>
+      <c r="D51" s="35">
+        <v>3.75</v>
+      </c>
       <c r="E51" s="3"/>
       <c r="F51" s="3"/>
       <c r="G51" s="3"/>
@@ -2412,7 +2421,7 @@
       <c r="C54" s="38"/>
       <c r="D54" s="39">
         <f>sum(D48:D52)</f>
-        <v>11.5</v>
+        <v>15.25</v>
       </c>
       <c r="E54" s="3"/>
       <c r="F54" s="3"/>

</xml_diff>

<commit_message>
create admin pages in figma
</commit_message>
<xml_diff>
--- a/Week_4/HealthCare Plus/Capstone Timesheet_Ripal Patel.xlsx
+++ b/Week_4/HealthCare Plus/Capstone Timesheet_Ripal Patel.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="44">
   <si>
     <t>Week_1</t>
   </si>
@@ -140,6 +140,9 @@
   </si>
   <si>
     <t>Add pages for patient, Doctors</t>
+  </si>
+  <si>
+    <t>Add pages for Admin</t>
   </si>
 </sst>
 </file>
@@ -2357,9 +2360,15 @@
     </row>
     <row r="52">
       <c r="A52" s="32"/>
-      <c r="B52" s="33"/>
-      <c r="C52" s="34"/>
-      <c r="D52" s="35"/>
+      <c r="B52" s="33" t="s">
+        <v>43</v>
+      </c>
+      <c r="C52" s="34">
+        <v>46063.0</v>
+      </c>
+      <c r="D52" s="35">
+        <v>3.5</v>
+      </c>
       <c r="E52" s="3"/>
       <c r="F52" s="3"/>
       <c r="G52" s="3"/>
@@ -2421,7 +2430,7 @@
       <c r="C54" s="38"/>
       <c r="D54" s="39">
         <f>sum(D48:D52)</f>
-        <v>15.25</v>
+        <v>18.75</v>
       </c>
       <c r="E54" s="3"/>
       <c r="F54" s="3"/>

</xml_diff>